<commit_message>
Daily slate 2026-06-16 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-14.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-14.xlsx
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E3" t="n">
         <v>61</v>
       </c>
       <c r="F3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G3" t="n">
-        <v>70.90000000000001</v>
+        <v>70.09999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="E4" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F4" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="G4" t="n">
-        <v>46.4</v>
+        <v>46.3</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F5" t="n">
         <v>13</v>
       </c>
       <c r="G5" t="n">
-        <v>58.1</v>
+        <v>59.4</v>
       </c>
     </row>
     <row r="6">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E7" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F7" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G7" t="n">
-        <v>53.1</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="8">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E9" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G9" t="n">
-        <v>55.2</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>944</v>
+        <v>1027</v>
       </c>
       <c r="E11" t="n">
-        <v>604</v>
+        <v>652</v>
       </c>
       <c r="F11" t="n">
-        <v>340</v>
+        <v>375</v>
       </c>
       <c r="G11" t="n">
-        <v>64</v>
+        <v>63.5</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="E12" t="n">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="F12" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G12" t="n">
-        <v>67.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>329</v>
+        <v>349</v>
       </c>
       <c r="E14" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F14" t="n">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="G14" t="n">
-        <v>24.9</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>385</v>
+        <v>409</v>
       </c>
       <c r="E15" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F15" t="n">
-        <v>322</v>
+        <v>339</v>
       </c>
       <c r="G15" t="n">
-        <v>16.4</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E16" t="n">
         <v>40</v>
       </c>
       <c r="F16" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G16" t="n">
-        <v>22.6</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3601</v>
+        <v>3966</v>
       </c>
       <c r="E17" t="n">
-        <v>840</v>
+        <v>939</v>
       </c>
       <c r="F17" t="n">
-        <v>2761</v>
+        <v>3027</v>
       </c>
       <c r="G17" t="n">
-        <v>23.3</v>
+        <v>23.7</v>
       </c>
     </row>
   </sheetData>
@@ -1540,16 +1540,16 @@
         <v>94</v>
       </c>
       <c r="D7" t="n">
-        <v>64</v>
+        <v>63.5</v>
       </c>
       <c r="E7" t="n">
-        <v>944</v>
+        <v>1027</v>
       </c>
       <c r="F7" t="n">
-        <v>67.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="H7" t="n">
         <v>56.9</v>
@@ -1558,28 +1558,28 @@
         <v>65</v>
       </c>
       <c r="J7" t="n">
-        <v>24.9</v>
+        <v>25.2</v>
       </c>
       <c r="K7" t="n">
-        <v>329</v>
+        <v>349</v>
       </c>
       <c r="L7" t="n">
-        <v>16.4</v>
+        <v>17.1</v>
       </c>
       <c r="M7" t="n">
-        <v>385</v>
+        <v>409</v>
       </c>
       <c r="N7" t="n">
-        <v>22.6</v>
+        <v>22.3</v>
       </c>
       <c r="O7" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="P7" t="n">
-        <v>23.3</v>
+        <v>23.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>3601</v>
+        <v>3966</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
@@ -1588,10 +1588,10 @@
         <v>140</v>
       </c>
       <c r="T7" t="n">
-        <v>46.4</v>
+        <v>46.3</v>
       </c>
       <c r="U7" t="n">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
@@ -1606,28 +1606,28 @@
         <v>303</v>
       </c>
       <c r="Z7" t="n">
-        <v>70.90000000000001</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="AA7" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AB7" t="n">
-        <v>58.1</v>
+        <v>59.4</v>
       </c>
       <c r="AC7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AD7" t="n">
-        <v>53.1</v>
+        <v>52.5</v>
       </c>
       <c r="AE7" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="AF7" t="n">
-        <v>55.2</v>
+        <v>55.6</v>
       </c>
       <c r="AG7" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>